<commit_message>
🤖 自动更新价格数据 2026-09-13 05:27:33
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D297"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,16 +5161,32 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C297" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D297" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B297" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C297" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D297" t="n">
+      <c r="B298" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C298" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D298" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-14 05:31:58
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,16 +5177,32 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C298" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D298" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B298" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C298" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D298" t="n">
+      <c r="B299" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C299" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D299" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-15 05:32:11
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D299"/>
+  <dimension ref="A1:D300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,16 +5193,32 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C299" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D299" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B299" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C299" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D299" t="n">
+      <c r="B300" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C300" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D300" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-16 05:24:42
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D300"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,16 +5209,32 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C300" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D300" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B300" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C300" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D300" t="n">
+      <c r="B301" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C301" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D301" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-17 05:33:27
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D301"/>
+  <dimension ref="A1:D302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,16 +5225,32 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C301" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D301" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B301" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C301" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D301" t="n">
+      <c r="B302" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C302" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D302" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-18 05:21:18
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D302"/>
+  <dimension ref="A1:D303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,16 +5241,32 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C302" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D302" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B302" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C302" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D302" t="n">
+      <c r="B303" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C303" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D303" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-19 05:13:24
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D303"/>
+  <dimension ref="A1:D304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,16 +5257,32 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C303" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D303" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B303" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C303" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D303" t="n">
+      <c r="B304" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C304" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D304" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-20 05:30:29
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D304"/>
+  <dimension ref="A1:D305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,16 +5273,32 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C304" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D304" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B304" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C304" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D304" t="n">
+      <c r="B305" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C305" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D305" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-21 05:35:35
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D305"/>
+  <dimension ref="A1:D306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,16 +5289,32 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C305" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D305" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B305" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C305" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D305" t="n">
+      <c r="B306" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C306" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D306" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-22 05:32:36
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D306"/>
+  <dimension ref="A1:D307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,16 +5305,32 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C306" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D306" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B306" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C306" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D306" t="n">
+      <c r="B307" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C307" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D307" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-23 05:20:30
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D307"/>
+  <dimension ref="A1:D308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,16 +5321,32 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C307" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D307" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B307" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C307" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D307" t="n">
+      <c r="B308" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C308" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D308" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-24 05:35:57
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D308"/>
+  <dimension ref="A1:D309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,16 +5337,32 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C308" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D308" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B308" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C308" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D308" t="n">
+      <c r="B309" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C309" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D309" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-25 05:32:54
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D309"/>
+  <dimension ref="A1:D310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,16 +5353,32 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C309" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D309" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B309" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C309" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D309" t="n">
+      <c r="B310" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C310" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D310" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-26 05:39:32
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D310"/>
+  <dimension ref="A1:D311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,16 +5369,32 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C310" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D310" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B310" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C310" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D310" t="n">
+      <c r="B311" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C311" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D311" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-27 05:55:42
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D311"/>
+  <dimension ref="A1:D312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,16 +5385,32 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C311" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D311" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B311" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C311" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D311" t="n">
+      <c r="B312" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C312" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D312" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-28 06:02:53
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D312"/>
+  <dimension ref="A1:D313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,16 +5401,32 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C312" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D312" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B312" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C312" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D312" t="n">
+      <c r="B313" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C313" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D313" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-29 06:20:28
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D313"/>
+  <dimension ref="A1:D314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,16 +5417,32 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C313" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D313" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B313" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C313" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D313" t="n">
+      <c r="B314" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C314" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D314" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-09-30 06:05:21
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,16 +5433,32 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C314" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D314" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B314" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C314" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D314" t="n">
+      <c r="B315" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C315" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D315" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-01 06:39:02
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D315"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,16 +5449,32 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C315" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D315" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B315" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C315" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D315" t="n">
+      <c r="B316" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C316" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D316" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-02 06:22:20
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D316"/>
+  <dimension ref="A1:D317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,16 +5465,32 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C316" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D316" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B316" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C316" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D316" t="n">
+      <c r="B317" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C317" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D317" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-03 05:51:56
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D317"/>
+  <dimension ref="A1:D318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,16 +5481,32 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C317" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D317" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B317" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C317" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D317" t="n">
+      <c r="B318" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C318" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D318" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-04 06:28:51
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D318"/>
+  <dimension ref="A1:D319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,16 +5497,32 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C318" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D318" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B318" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C318" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D318" t="n">
+      <c r="B319" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C319" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D319" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-05 06:21:45
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D319"/>
+  <dimension ref="A1:D320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,16 +5513,32 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C319" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D319" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B319" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C319" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D319" t="n">
+      <c r="B320" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C320" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D320" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-06 06:57:34
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D320"/>
+  <dimension ref="A1:D321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,16 +5529,32 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C320" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D320" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B320" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C320" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D320" t="n">
+      <c r="B321" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C321" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D321" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-07 06:38:50
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D321"/>
+  <dimension ref="A1:D322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,16 +5545,32 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C321" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D321" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B321" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C321" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D321" t="n">
+      <c r="B322" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C322" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D322" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-08 06:45:21
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D322"/>
+  <dimension ref="A1:D323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,16 +5561,32 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C322" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D322" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B322" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C322" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D322" t="n">
+      <c r="B323" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C323" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D323" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-09 06:53:10
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D323"/>
+  <dimension ref="A1:D324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,7 +5561,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -5577,16 +5577,32 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C323" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D323" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B323" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C323" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D323" t="n">
+      <c r="B324" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C324" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D324" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-10 06:29:33
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D324"/>
+  <dimension ref="A1:D325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,7 +5561,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -5577,7 +5577,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -5593,16 +5593,32 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C324" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D324" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B324" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C324" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D324" t="n">
+      <c r="B325" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C325" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D325" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-11 06:35:21
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D325"/>
+  <dimension ref="A1:D326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,7 +5561,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -5577,7 +5577,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -5593,7 +5593,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -5609,16 +5609,32 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C325" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D325" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B325" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C325" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D325" t="n">
+      <c r="B326" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C326" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D326" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-12 06:40:40
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D326"/>
+  <dimension ref="A1:D327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,7 +5561,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -5577,7 +5577,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -5593,7 +5593,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -5609,7 +5609,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -5625,16 +5625,32 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C326" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D326" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B326" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C326" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D326" t="n">
+      <c r="B327" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C327" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D327" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-13 07:10:51
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D327"/>
+  <dimension ref="A1:D328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -4729,7 +4729,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -4745,7 +4745,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-17</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -4761,7 +4761,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -4777,7 +4777,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -4793,7 +4793,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -4809,7 +4809,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -4825,7 +4825,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>2026-01-11</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -4841,7 +4841,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -4857,7 +4857,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -4873,7 +4873,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -4889,7 +4889,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -4905,7 +4905,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -4921,7 +4921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -4937,7 +4937,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -4953,7 +4953,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -4969,7 +4969,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -4985,7 +4985,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5001,7 +5001,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5017,7 +5017,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5033,7 +5033,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5049,7 +5049,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5065,7 +5065,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5081,7 +5081,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5097,7 +5097,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5113,7 +5113,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-25</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5129,7 +5129,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5145,7 +5145,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5161,7 +5161,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5177,7 +5177,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5193,7 +5193,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5209,7 +5209,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5225,7 +5225,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5241,7 +5241,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5257,7 +5257,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5273,7 +5273,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5289,7 +5289,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5305,7 +5305,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5321,7 +5321,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5337,7 +5337,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5353,7 +5353,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5369,7 +5369,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -5385,7 +5385,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -5401,7 +5401,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -5417,7 +5417,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -5433,7 +5433,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -5449,7 +5449,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -5465,7 +5465,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -5481,7 +5481,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -5497,7 +5497,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -5513,7 +5513,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -5529,7 +5529,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -5545,7 +5545,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -5561,7 +5561,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -5577,7 +5577,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -5593,7 +5593,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -5609,7 +5609,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -5625,7 +5625,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B326" t="n">
@@ -5641,16 +5641,32 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C327" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D327" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="B327" t="n">
-        <v>783.5</v>
-      </c>
-      <c r="C327" t="n">
-        <v>1112</v>
-      </c>
-      <c r="D327" t="n">
+      <c r="B328" t="n">
+        <v>783.5</v>
+      </c>
+      <c r="C328" t="n">
+        <v>1112</v>
+      </c>
+      <c r="D328" t="n">
         <v>3610</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 自动更新价格数据 2026-10-14 05:34:19
</commit_message>
<xml_diff>
--- a/商品价格数据.xlsx
+++ b/商品价格数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D328"/>
+  <dimension ref="A1:D329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -537,7 +537,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -553,7 +553,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -569,7 +569,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -585,7 +585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -601,7 +601,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -617,7 +617,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -665,7 +665,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -681,7 +681,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -697,7 +697,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -713,7 +713,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -729,7 +729,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -761,7 +761,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -777,7 +777,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -793,7 +793,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -809,7 +809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -825,7 +825,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -841,7 +841,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -857,7 +857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -873,7 +873,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -889,7 +889,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -905,7 +905,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -921,7 +921,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -937,7 +937,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -953,7 +953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -969,7 +969,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -985,7 +985,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1001,7 +1001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1017,7 +1017,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1033,7 +1033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1049,7 +1049,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1065,7 +1065,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1081,7 +1081,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1097,7 +1097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1113,7 +1113,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1129,7 +1129,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1145,7 +1145,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1161,7 +1161,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1193,7 +1193,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1209,7 +1209,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1225,7 +1225,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1241,7 +1241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1257,7 +1257,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1273,7 +1273,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1289,7 +1289,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1305,7 +1305,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1321,7 +1321,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1337,7 +1337,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1353,7 +1353,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1369,7 +1369,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1385,7 +1385,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1401,7 +1401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1417,7 +1417,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1433,7 +1433,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1449,7 +1449,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1465,7 +1465,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1481,7 +1481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1497,7 +1497,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1513,7 +1513,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1529,7 +1529,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1545,7 +1545,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1561,7 +1561,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1577,7 +1577,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1593,7 +1593,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1609,7 +1609,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1625,7 +1625,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1641,7 +1641,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1657,7 +1657,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1673,7 +1673,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1689,7 +1689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1705,7 +1705,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1721,7 +1721,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1737,7 +1737,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1753,7 +1753,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1769,7 +1769,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1785,7 +1785,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1801,7 +1801,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1817,7 +1817,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1833,7 +1833,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1849,7 +1849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1865,7 +1865,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1881,7 +1881,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1897,7 +1897,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1913,7 +1913,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1929,7 +1929,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1945,7 +1945,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1961,7 +1961,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1977,7 +1977,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1993,7 +1993,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2009,7 +2009,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2025,7 +2025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2041,7 +2041,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2057,7 +2057,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2073,7 +2073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2089,7 +2089,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2105,7 +2105,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2121,7 +2121,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2137,7 +2137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2153,7 +2153,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2169,7 +2169,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2185,7 +2185,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2201,7 +2201,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2217,7 +2217,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2233,7 +2233,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2249,7 +2249,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2265,7 +2265,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2281,7 +2281,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2297,7 +2297,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2313,7 +2313,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2329,7 +2329,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2345,7 +2345,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2361,7 +2361,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2377,7 +2377,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2393,7 +2393,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2409,7 +2409,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2425,7 +2425,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2441,7 +2441,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2457,7 +2457,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2473,7 +2473,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2489,7 +2489,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2505,7 +2505,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2521,7 +2521,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2537,7 +2537,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2553,7 +2553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2569,7 +2569,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2585,7 +2585,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2601,7 +2601,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2617,7 +2617,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2633,7 +2633,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2649,7 +2649,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2665,7 +2665,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2681,7 +2681,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2697,7 +2697,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -2713,7 +2713,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -2729,7 +2729,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -2745,7 +2745,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -2761,7 +2761,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -2777,7 +2777,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -2793,7 +2793,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -2809,7 +2809,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -2825,7 +2825,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -2841,7 +2841,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -2857,7 +2857,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -2873,7 +2873,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -2889,7 +2889,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -2905,7 +2905,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -2921,7 +2921,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2937,7 +2937,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2953,7 +2953,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2969,7 +2969,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2985,7 +2985,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3001,7 +3001,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3017,7 +3017,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3033,7 +3033,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3049,7 +3049,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3065,7 +3065,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3081,7 +3081,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3097,7 +3097,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3113,7 +3113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3129,7 +3129,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3145,7 +3145,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3161,7 +3161,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3177,7 +3177,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3193,7 +3193,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3209,7 +3209,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3225,7 +3225,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3241,7 +3241,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3257,7 +3257,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3273,7 +3273,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3289,7 +3289,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3305,7 +3305,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3321,7 +3321,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3337,7 +3337,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3353,7 +3353,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3369,7 +3369,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3385,7 +3385,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3401,7 +3401,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3417,7 +3417,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3433,7 +3433,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3449,7 +3449,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3465,7 +3465,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3481,7 +3481,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3497,7 +3497,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3513,7 +3513,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3529,7 +3529,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3545,7 +3545,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3561,7 +3561,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3577,7 +3577,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3593,7 +3593,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -3609,7 +3609,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -3625,7 +3625,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -3641,7 +3641,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -3657,7 +3657,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -3673,7 +3673,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -3689,7 +3689,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -3705,7 +3705,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -3721,7 +3721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -3737,7 +3737,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -3753,7 +3753,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -3769,7 +3769,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -3785,7 +3785,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -3801,7 +3801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -3817,7 +3817,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -3833,7 +3833,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -3849,7 +3849,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -3865,7 +3865,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -3881,7 +3881,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -3897,7 +3897,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -3913,7 +3913,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -3929,7 +3929,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -3945,7 +3945,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -3961,7 +3961,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -3977,7 +3977,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -3993,7 +3993,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4009,7 +4009,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4025,7 +4025,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4041,7 +4041,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4057,7 +4057,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4073,7 +4073,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4089,7 +4089,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4105,7 +4105,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4121,7 +4121,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4137,7 +4137,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4153,7 +4153,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4169,7 +4169,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4185,7 +4185,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4201,7 +4201,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4217,7 +4217,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4233,7 +4233,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4249,7 +4249,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4265,7 +4265,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4281,7 +4281,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4297,7 +4297,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4313,7 +4313,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4329,7 +4329,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4345,7 +4345,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4361,7 +4361,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4377,7 +4377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4393,7 +4393,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4409,7 +4409,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-08</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4425,7 +4425,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4441,7 +4441,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4457,7 +4457,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4473,7 +4473,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -4489,7 +4489,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -4505,7 +4505,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -4521,7 +4521,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -4537,7 +4537,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -4553,7 +4553,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -4569,7 +4569,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -4585,7 +4585,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -4601,7 +4601,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -4617,7 +4617,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -4633,7 +4633,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -4649,7 +4649,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -4665,7 +4665,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -4681,7 +4681,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -4697,7 +4697,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -4713,7 +4713,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-       